<commit_message>
Copy all files from TIM LEAF and override from main
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_PWR_DH.xlsx
+++ b/SubRES_TMPL/SubRES_PWR_DH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SubRES_TMPL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olex\Documents\MANRID\ResLab\Modelling\TIMES\TIMES-IE\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208FE9C8-B0EB-44E2-BA58-6C08F43EBA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25CBD38A-783F-4731-9BFB-01C5E75B76B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -986,6 +986,9 @@
     <t>Output Commodity</t>
   </si>
   <si>
+    <t>VAROM</t>
+  </si>
+  <si>
     <t>CAP2ACT</t>
   </si>
   <si>
@@ -1004,6 +1007,9 @@
     <t>Investment Cost</t>
   </si>
   <si>
+    <t>Variable O&amp;M Cost</t>
+  </si>
+  <si>
     <t>New Processes</t>
   </si>
   <si>
@@ -1167,12 +1173,6 @@
   </si>
   <si>
     <t>MEUR2018</t>
-  </si>
-  <si>
-    <t>FIXOM</t>
-  </si>
-  <si>
-    <t>Fixed O&amp;M Cost</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1436,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1529,7 +1529,6 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="4" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1870,7 +1869,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="IEA Data"/>
@@ -2005,9 +2004,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2045,9 +2044,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2080,9 +2079,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2115,9 +2131,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2728,12 +2761,12 @@
       <c r="Z15" s="25"/>
     </row>
     <row r="16" spans="1:26" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="42" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
+      <c r="A16" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
@@ -2815,13 +2848,13 @@
     </row>
     <row r="19" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="41" t="s">
-        <v>97</v>
-      </c>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
+        <v>88</v>
+      </c>
+      <c r="B19" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
       <c r="E19" s="33"/>
       <c r="F19" s="33"/>
       <c r="G19" s="34"/>
@@ -2847,13 +2880,13 @@
     </row>
     <row r="20" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="B20" s="41" t="s">
-        <v>98</v>
-      </c>
-      <c r="C20" s="41"/>
-      <c r="D20" s="41"/>
+        <v>89</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
       <c r="E20" s="33"/>
       <c r="F20" s="33"/>
       <c r="G20" s="34"/>
@@ -2879,10 +2912,10 @@
     </row>
     <row r="21" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="32" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C21" s="35"/>
       <c r="D21" s="35"/>
@@ -2939,13 +2972,13 @@
     </row>
     <row r="23" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B23" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
+        <v>91</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
       <c r="E23" s="25"/>
       <c r="F23" s="25"/>
       <c r="G23" s="25"/>
@@ -2971,11 +3004,11 @@
     </row>
     <row r="24" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32"/>
-      <c r="B24" s="41" t="s">
-        <v>101</v>
-      </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
+      <c r="B24" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
       <c r="E24" s="25"/>
       <c r="F24" s="25"/>
       <c r="G24" s="25"/>
@@ -3029,13 +3062,13 @@
     </row>
     <row r="26" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="B26" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
+        <v>92</v>
+      </c>
+      <c r="B26" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
       <c r="E26" s="25"/>
       <c r="F26" s="25"/>
       <c r="G26" s="25"/>
@@ -3061,11 +3094,11 @@
     </row>
     <row r="27" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="32"/>
-      <c r="B27" s="41" t="s">
-        <v>101</v>
-      </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
+      <c r="B27" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
       <c r="E27" s="25"/>
       <c r="F27" s="25"/>
       <c r="G27" s="25"/>
@@ -3119,7 +3152,7 @@
     </row>
     <row r="29" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="32" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B29" s="36">
         <v>1</v>
@@ -3151,13 +3184,13 @@
     </row>
     <row r="30" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="B30" s="43" t="s">
-        <v>93</v>
-      </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
+        <v>94</v>
+      </c>
+      <c r="B30" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
       <c r="E30" s="37"/>
       <c r="F30" s="37"/>
       <c r="G30" s="25"/>
@@ -3183,13 +3216,13 @@
     </row>
     <row r="31" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="B31" s="41" t="s">
-        <v>95</v>
-      </c>
-      <c r="C31" s="41"/>
-      <c r="D31" s="41"/>
+        <v>96</v>
+      </c>
+      <c r="B31" s="40" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="40"/>
+      <c r="D31" s="40"/>
       <c r="E31" s="37"/>
       <c r="F31" s="37"/>
       <c r="G31" s="25"/>
@@ -3216,7 +3249,7 @@
     <row r="32" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="38"/>
       <c r="B32" s="39" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C32" s="38"/>
       <c r="D32" s="38"/>
@@ -5173,7 +5206,7 @@
   <sheetData>
     <row r="1" spans="2:25" ht="18" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1"/>
       <c r="G1" s="1" t="s">
@@ -5191,7 +5224,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>3</v>
@@ -5200,10 +5233,10 @@
         <v>4</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>15</v>
@@ -5215,19 +5248,19 @@
         <v>5</v>
       </c>
       <c r="K2" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="M2" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="O2" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>103</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>16</v>
@@ -5269,31 +5302,31 @@
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H3" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>45</v>
-      </c>
       <c r="L3" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O3" s="10" t="s">
-        <v>104</v>
+        <v>49</v>
       </c>
       <c r="R3" s="7" t="s">
         <v>31</v>
@@ -5322,22 +5355,22 @@
     </row>
     <row r="4" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B4" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F4">
         <v>2020</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H4">
         <v>2022</v>
@@ -5361,12 +5394,8 @@
       <c r="N4" s="13">
         <v>5</v>
       </c>
-      <c r="O4" s="40">
-        <f>L4*7%</f>
-        <v>2.1678999999999999</v>
-      </c>
       <c r="R4" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S4" s="13" t="str">
         <f>DH_Grid_Extension!B4</f>
@@ -5377,35 +5406,35 @@
         <v>District Heating Network Extension - S1</v>
       </c>
       <c r="U4" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="V4" s="13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="W4" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="X4" s="8"/>
       <c r="Y4" s="8"/>
     </row>
     <row r="5" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B5" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F5">
         <v>2020</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H5">
         <v>2022</v>
@@ -5429,12 +5458,8 @@
       <c r="N5" s="13">
         <v>5</v>
       </c>
-      <c r="O5" s="40">
-        <f t="shared" ref="O5:O6" si="0">L5*7%</f>
-        <v>3.9158000000000004</v>
-      </c>
       <c r="R5" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S5" s="13" t="str">
         <f>DH_Grid_Extension!B5</f>
@@ -5445,33 +5470,33 @@
         <v>District Heating Network Extension - S2</v>
       </c>
       <c r="U5" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="V5" s="13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="W5" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B6" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F6">
         <v>2020</v>
       </c>
       <c r="G6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H6">
         <v>2022</v>
@@ -5495,12 +5520,8 @@
       <c r="N6" s="13">
         <v>5</v>
       </c>
-      <c r="O6" s="40">
-        <f t="shared" si="0"/>
-        <v>6.8866000000000005</v>
-      </c>
       <c r="R6" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S6" s="13" t="str">
         <f>DH_Grid_Extension!B6</f>
@@ -5511,13 +5532,13 @@
         <v>District Heating Network Extension - S3</v>
       </c>
       <c r="U6" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="V6" s="13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="W6" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="2:25" x14ac:dyDescent="0.2">
@@ -5638,41 +5659,41 @@
       <c r="B3" s="14"/>
       <c r="C3" s="15"/>
       <c r="D3" s="16" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B4" s="14"/>
       <c r="C4" s="14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="B5" s="15" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C5" s="14">
         <v>311.65399600000001</v>
@@ -5693,7 +5714,7 @@
     </row>
     <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="B6" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C6" s="19">
         <v>2.9555506715861044E-3</v>
@@ -5714,7 +5735,7 @@
     </row>
     <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C7" s="21"/>
       <c r="D7" s="21">
@@ -5733,7 +5754,7 @@
     </row>
     <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="B8" s="15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14">
@@ -5752,7 +5773,7 @@
     </row>
     <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="B9" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="22">
@@ -5784,7 +5805,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" s="23" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C11" s="23"/>
       <c r="D11" s="23"/>

</xml_diff>